<commit_message>
Actualizacao da pagina sobre Feiras
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -414,55 +414,739 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>02-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3918786000010555084</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>TOPELANE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>02-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>3918786000010555030</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>30-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>3918786000010552123</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>3918786000010552121</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>3918786000010552119</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>01-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3918786000010538052</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MOCONE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Belo Simao</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>02-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>3918786000010422028</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Nacala Porto</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Otilia Passiel</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>3918786000010407006</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>3918786000010405032</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>16-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>3918786000010405030</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>05-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3918786000010405028</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>3918786000010405026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>03-Jun-2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>3918786000010320010</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Monapo</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -729,13 +1413,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF2606EE-5354-442E-B5C4-A0481178E321}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66617C0E-440C-4D68-9BA6-A5696479021E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87A958B1-8CE5-4FFA-99D3-2FAE30873002}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49E8C722-AECD-44EF-9212-5A6676B06D05}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEF0F17B-CE35-47E1-B2C7-16462AE8A825}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94636A10-6C1C-4E79-A22D-B30561F90498}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao graficos das feiras
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -414,7 +414,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -424,37 +424,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010555084</t>
+          <t>3918786000010579063</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -471,47 +471,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Paulo Alexandre</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TOPELANE</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sessão_3</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Costa Marques</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>03-Jun-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3918786000010555030</t>
+          <t>3918786000010579061</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3918786000010552123</t>
+          <t>3918786000010579059</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3918786000010552121</t>
+          <t>3918786000010573006</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -652,17 +652,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3918786000010552119</t>
+          <t>3918786000010555084</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3918786000010538052</t>
+          <t>3918786000010555030</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -756,7 +756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -766,17 +766,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MOCONE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Belo Simao</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -786,22 +786,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>02-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3918786000010422028</t>
+          <t>3918786000010552123</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Otilia Passiel</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3918786000010407006</t>
+          <t>3918786000010552121</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -880,17 +880,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -900,17 +900,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3918786000010405032</t>
+          <t>3918786000010552119</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -937,12 +937,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3918786000010405030</t>
+          <t>3918786000010538052</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MOCONE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Belo Simao</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1014,22 +1014,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>05-Jun-2026</t>
+          <t>02-Jun-2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3918786000010405028</t>
+          <t>3918786000010422028</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1041,47 +1041,47 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Otilia Passiel</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>RAMIANE</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Sessão_1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Costa Marques</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>04-Jun-2026</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3918786000010405026</t>
+          <t>3918786000010407006</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1098,55 +1098,283 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>3918786000010405032</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>16-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>3918786000010405030</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>05-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3918786000010405028</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>3918786000010405026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>TOPELANE</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>03-Jun-2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>3918786000010320010</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Monapo</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1155,271 +1383,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
-    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66617C0E-440C-4D68-9BA6-A5696479021E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49E8C722-AECD-44EF-9212-5A6676B06D05}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94636A10-6C1C-4E79-A22D-B30561F90498}"/>
 </file>
</xml_diff>

<commit_message>
Actualização das 4 sessao
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -414,7 +414,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -424,7 +424,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010638034</t>
+          <t>3918786000010652028</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -481,17 +481,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -501,17 +501,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>16-Jul-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3918786000010611006</t>
+          <t>3918786000010640095</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -538,17 +538,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3918786000010611004</t>
+          <t>3918786000010639055</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -595,17 +595,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3918786000010611002</t>
+          <t>3918786000010638034</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -652,37 +652,37 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3918786000010579063</t>
+          <t>3918786000010611006</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -709,37 +709,37 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>03-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3918786000010579061</t>
+          <t>3918786000010611004</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -756,7 +756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -766,17 +766,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -786,17 +786,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3918786000010579059</t>
+          <t>3918786000010611002</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -833,27 +833,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3918786000010573006</t>
+          <t>3918786000010579063</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -880,37 +880,37 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>03-Jun-2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3918786000010555084</t>
+          <t>3918786000010579061</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -962,12 +962,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3918786000010555030</t>
+          <t>3918786000010579059</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -994,17 +994,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3918786000010552123</t>
+          <t>3918786000010573006</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1051,17 +1051,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1071,17 +1071,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3918786000010552121</t>
+          <t>3918786000010555084</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1108,17 +1108,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1128,17 +1128,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3918786000010552119</t>
+          <t>3918786000010555030</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3918786000010538052</t>
+          <t>3918786000010552123</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1212,7 +1212,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MOCONE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Belo Simao</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1242,22 +1242,22 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>02-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3918786000010422028</t>
+          <t>3918786000010552121</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1269,7 +1269,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1279,17 +1279,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Otilia Passiel</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3918786000010407006</t>
+          <t>3918786000010552119</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1356,17 +1356,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3918786000010405032</t>
+          <t>3918786000010538052</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1383,7 +1383,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1393,17 +1393,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MOCONE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Belo Simao</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1413,22 +1413,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>02-Jun-2026</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3918786000010405030</t>
+          <t>3918786000010422028</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1450,17 +1450,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Otilia Passiel</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>05-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3918786000010405028</t>
+          <t>3918786000010407006</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1497,7 +1497,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1527,17 +1527,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>3918786000010405026</t>
+          <t>3918786000010405032</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1554,55 +1554,226 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>16-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>3918786000010405030</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>05-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>3918786000010405028</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>3918786000010405026</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>TOPELANE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>03-Jun-2026</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>3918786000010320010</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Monapo</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1869,13 +2040,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8DACBAB-C254-412E-891B-C6C4287CB82D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20790C72-730F-4A78-BFB6-431DA486FB12}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6E93D27-0500-49A1-B955-D701B2354559}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B9984D60-14C6-4970-BF43-F56F8CC769E1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8ACD27-436A-4670-AECA-6D20BA160015}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{71164310-56A2-4F84-9B29-A0E595EDE16E}"/>
 </file>
</xml_diff>